<commit_message>
Auto backup: 2026-05-24_ 2:19:26.15
</commit_message>
<xml_diff>
--- a/plans/dddd.xlsx
+++ b/plans/dddd.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -63,8 +63,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00EBFDEB"/>
+        <bgColor rgb="00EBFDEB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF0FF"/>
+        <bgColor rgb="00FBF0FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6DCFA"/>
+        <bgColor rgb="00F6DCFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4FADC"/>
+        <bgColor rgb="00F4FADC"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,12 +98,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -686,37 +707,37 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>NEONSAT1</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NEONSAT12</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>NEW_ACTIVITY</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>305</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -760,74 +781,111 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>SPACEEYE-T1</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>NEONSAT12</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>NEW_ACTIVITY</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>307</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>NEONSAT1A</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>NEONSAT13</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>NEW_ACTIVITY</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>308</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>NEONSAT122</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>NEW_ACTIVITY</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>309</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>